<commit_message>
fix(excel & dicom): patch v2.1.6 minor fix with 25-col template styling and dicom test connection
</commit_message>
<xml_diff>
--- a/Daftar_Radiologi/template.xlsx
+++ b/Daftar_Radiologi/template.xlsx
@@ -40,22 +40,22 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00E0F2F1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="10"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,24 +64,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00004D40"/>
-        <bgColor rgb="00004D40"/>
+        <fgColor rgb="002F6EBA"/>
+        <bgColor rgb="002F6EBA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000695C"/>
-        <bgColor rgb="0000695C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FACC15"/>
-        <bgColor rgb="00FACC15"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -91,33 +85,46 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00204E85"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00204E85"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00204E85"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00204E85"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -515,10 +522,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -552,164 +559,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -750,10 +753,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -787,164 +790,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -985,10 +984,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1022,164 +1021,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1220,10 +1215,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1257,164 +1252,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1455,10 +1446,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1492,164 +1483,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1690,10 +1677,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1727,164 +1714,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1925,10 +1908,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1962,164 +1945,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2160,10 +2139,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2197,164 +2176,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2395,10 +2370,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2432,164 +2407,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2630,10 +2601,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2667,164 +2638,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2865,10 +2832,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2902,164 +2869,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3100,10 +3063,10 @@
     <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUKU DAFTAR RADIOLOGI {SINGKATAN KLINIK}</t>
+          <t>BUKU DAFTAR RADIOLOGI KKBBS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3137,164 +3100,160 @@
           <t>KEMENTERIAN KESIHATAN MALAYSIA — REKOD PENDAFTARAN PESAKIT (PER.SS-RA 101)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TARIKH</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>LMP</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bil Kes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nombor X-ray</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Nombor Kad Pengenalan /Pasport</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>UMUR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>JANTINA</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>W/NEGARA</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>KAKITANGAN KERAJAAN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>BANGSA</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>ALAMAT</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>JENIS</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>BAHAGIAN</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>LATERALLY</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KLINIK</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KATEGORI</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>CD/FILEM</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>TOTAL EXPOSE</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>TOTAL REJECT</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>FILEM / CD</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>PERSON TAKEN</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>